<commit_message>
Fixes a minor naming inconsistency
</commit_message>
<xml_diff>
--- a/MasterSheet.xlsx
+++ b/MasterSheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\10DOT\Deliverable1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\10DOT\Deliverable1\10DOT_SubmissionPackage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768995F8-26C9-46AB-AA1D-C60DFE3B0504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D71A528-EFB6-47BF-92CF-D9869F21EE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12840" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RAW_DATA" sheetId="1" r:id="rId1"/>
@@ -10438,9 +10438,6 @@
     <t>Technical knowledge before interaction</t>
   </si>
   <si>
-    <t>Objective Metrics</t>
-  </si>
-  <si>
     <t>Technical Behavior</t>
   </si>
   <si>
@@ -10776,6 +10773,9 @@
   </si>
   <si>
     <t>ABSTRACT (Relative)</t>
+  </si>
+  <si>
+    <t>Objective Sys. Properties</t>
   </si>
 </sst>
 </file>
@@ -11186,7 +11186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -11273,8 +11273,20 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -11287,20 +11299,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -43828,10 +43829,10 @@
       <c r="D601" s="8" t="s">
         <v>3340</v>
       </c>
-      <c r="E601" s="36" t="s">
+      <c r="E601" s="48" t="s">
         <v>3341</v>
       </c>
-      <c r="F601" s="37"/>
+      <c r="F601" s="49"/>
       <c r="G601" s="8"/>
       <c r="H601" s="7">
         <v>1135</v>
@@ -61889,16 +61890,16 @@
         <v>3384</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>3513</v>
+        <v>3512</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>3413</v>
       </c>
       <c r="E8" s="14" t="s">
+        <v>3513</v>
+      </c>
+      <c r="F8" s="20" t="s">
         <v>3514</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>3515</v>
       </c>
       <c r="G8" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B8 ) &gt; 0, "OK", "KO" )</f>
@@ -61910,7 +61911,7 @@
         <v>3375</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>3517</v>
+        <v>3516</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>3413</v>
@@ -61919,7 +61920,7 @@
         <v>3429</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>3518</v>
+        <v>3517</v>
       </c>
       <c r="G9" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B9 ) &gt; 0, "OK", "KO" )</f>
@@ -62036,7 +62037,7 @@
         <v>3368</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>3556</v>
+        <v>3555</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>3432</v>
@@ -62120,16 +62121,16 @@
         <v>3384</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>3510</v>
+        <v>3509</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>3432</v>
       </c>
       <c r="E19" s="14" t="s">
+        <v>3510</v>
+      </c>
+      <c r="F19" s="20" t="s">
         <v>3511</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>3512</v>
       </c>
       <c r="G19" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B19 ) &gt; 0, "OK", "KO" )</f>
@@ -62143,14 +62144,14 @@
       <c r="C20" s="14" t="s">
         <v>3435</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="50" t="s">
         <v>3432</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>3436</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>3516</v>
+        <v>3515</v>
       </c>
       <c r="G20" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B20 ) &gt; 0, "OK", "KO" )</f>
@@ -62162,7 +62163,7 @@
         <v>3376</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>3522</v>
+        <v>3521</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>3432</v>
@@ -62171,7 +62172,7 @@
         <v>3439</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>3523</v>
+        <v>3522</v>
       </c>
       <c r="G21" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B21 ) &gt; 0, "OK", "KO" )</f>
@@ -62297,7 +62298,7 @@
         <v>3450</v>
       </c>
       <c r="F27" s="20" t="s">
-        <v>3508</v>
+        <v>3507</v>
       </c>
       <c r="G27" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B27 ) &gt; 0, "OK", "KO" )</f>
@@ -62318,7 +62319,7 @@
         <v>3457</v>
       </c>
       <c r="F28" s="20" t="s">
-        <v>3509</v>
+        <v>3508</v>
       </c>
       <c r="G28" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B28 ) &gt; 0, "OK", "KO" )</f>
@@ -62330,7 +62331,7 @@
         <v>3387</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>3524</v>
+        <v>3523</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>3449</v>
@@ -62339,7 +62340,7 @@
         <v>3457</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>3525</v>
+        <v>3524</v>
       </c>
       <c r="G29" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B29 ) &gt; 0, "OK", "KO" )</f>
@@ -62351,16 +62352,16 @@
         <v>3376</v>
       </c>
       <c r="C30" s="14" t="s">
+        <v>3468</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E30" s="14" t="s">
         <v>3469</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E30" s="14" t="s">
+      <c r="F30" s="20" t="s">
         <v>3470</v>
-      </c>
-      <c r="F30" s="20" t="s">
-        <v>3471</v>
       </c>
       <c r="G30" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B30 ) &gt; 0, "OK", "KO" )</f>
@@ -62372,16 +62373,16 @@
         <v>3354</v>
       </c>
       <c r="C31" s="14" t="s">
+        <v>3468</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E31" s="14" t="s">
         <v>3469</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E31" s="14" t="s">
+      <c r="F31" s="20" t="s">
         <v>3470</v>
-      </c>
-      <c r="F31" s="20" t="s">
-        <v>3471</v>
       </c>
       <c r="G31" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B31 ) &gt; 0, "OK", "KO" )</f>
@@ -62393,16 +62394,16 @@
         <v>3395</v>
       </c>
       <c r="C32" s="14" t="s">
+        <v>3468</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>3469</v>
       </c>
-      <c r="D32" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E32" s="14" t="s">
+      <c r="F32" s="20" t="s">
         <v>3470</v>
-      </c>
-      <c r="F32" s="20" t="s">
-        <v>3471</v>
       </c>
       <c r="G32" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B32 ) &gt; 0, "OK", "KO" )</f>
@@ -62414,16 +62415,16 @@
         <v>3395</v>
       </c>
       <c r="C33" s="14" t="s">
+        <v>3471</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>3469</v>
+      </c>
+      <c r="F33" s="20" t="s">
         <v>3472</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>3470</v>
-      </c>
-      <c r="F33" s="20" t="s">
-        <v>3473</v>
       </c>
       <c r="G33" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B33 ) &gt; 0, "OK", "KO" )</f>
@@ -62435,16 +62436,16 @@
         <v>3376</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>3519</v>
+        <v>3518</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>3463</v>
+        <v>3575</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>3466</v>
+        <v>3465</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>3557</v>
+        <v>3556</v>
       </c>
       <c r="G34" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B34 ) &gt; 0, "OK", "KO" )</f>
@@ -62456,16 +62457,16 @@
         <v>3376</v>
       </c>
       <c r="C35" s="14" t="s">
+        <v>3519</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>3469</v>
+      </c>
+      <c r="F35" s="20" t="s">
         <v>3520</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>3470</v>
-      </c>
-      <c r="F35" s="20" t="s">
-        <v>3521</v>
       </c>
       <c r="G35" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B35 ) &gt; 0, "OK", "KO" )</f>
@@ -62477,16 +62478,16 @@
         <v>3395</v>
       </c>
       <c r="C36" s="14" t="s">
+        <v>3473</v>
+      </c>
+      <c r="D36" s="14" t="s">
         <v>3474</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="E36" s="14" t="s">
         <v>3475</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="F36" s="20" t="s">
         <v>3476</v>
-      </c>
-      <c r="F36" s="20" t="s">
-        <v>3477</v>
       </c>
       <c r="G36" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B36 ) &gt; 0, "OK", "KO" )</f>
@@ -62498,16 +62499,16 @@
         <v>3370</v>
       </c>
       <c r="C37" s="14" t="s">
+        <v>3473</v>
+      </c>
+      <c r="D37" s="14" t="s">
         <v>3474</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="E37" s="14" t="s">
         <v>3475</v>
       </c>
-      <c r="E37" s="14" t="s">
+      <c r="F37" s="20" t="s">
         <v>3476</v>
-      </c>
-      <c r="F37" s="20" t="s">
-        <v>3477</v>
       </c>
       <c r="G37" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B37 ) &gt; 0, "OK", "KO" )</f>
@@ -62519,16 +62520,16 @@
         <v>3395</v>
       </c>
       <c r="C38" s="14" t="s">
+        <v>3477</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F38" s="20" t="s">
         <v>3478</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F38" s="20" t="s">
-        <v>3479</v>
       </c>
       <c r="G38" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B38 ) &gt; 0, "OK", "KO" )</f>
@@ -62540,16 +62541,16 @@
         <v>3369</v>
       </c>
       <c r="C39" s="14" t="s">
+        <v>3477</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F39" s="20" t="s">
         <v>3478</v>
-      </c>
-      <c r="D39" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F39" s="20" t="s">
-        <v>3479</v>
       </c>
       <c r="G39" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B39 ) &gt; 0, "OK", "KO" )</f>
@@ -62561,16 +62562,16 @@
         <v>3400</v>
       </c>
       <c r="C40" s="14" t="s">
+        <v>3477</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F40" s="20" t="s">
         <v>3478</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F40" s="20" t="s">
-        <v>3479</v>
       </c>
       <c r="G40" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B40 ) &gt; 0, "OK", "KO" )</f>
@@ -62582,16 +62583,16 @@
         <v>3391</v>
       </c>
       <c r="C41" s="14" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F41" s="20" t="s">
         <v>3480</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F41" s="20" t="s">
-        <v>3481</v>
       </c>
       <c r="G41" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B41 ) &gt; 0, "OK", "KO" )</f>
@@ -62603,16 +62604,16 @@
         <v>3364</v>
       </c>
       <c r="C42" s="14" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F42" s="20" t="s">
         <v>3480</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E42" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F42" s="20" t="s">
-        <v>3481</v>
       </c>
       <c r="G42" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B42 ) &gt; 0, "OK", "KO" )</f>
@@ -62624,16 +62625,16 @@
         <v>3395</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F43" s="20" t="s">
         <v>3480</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F43" s="20" t="s">
-        <v>3481</v>
       </c>
       <c r="G43" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B43 ) &gt; 0, "OK", "KO" )</f>
@@ -62642,19 +62643,19 @@
     </row>
     <row r="44" spans="2:7">
       <c r="B44" s="14" t="s">
-        <v>3482</v>
+        <v>3481</v>
       </c>
       <c r="C44" s="14" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F44" s="20" t="s">
         <v>3480</v>
-      </c>
-      <c r="D44" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E44" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F44" s="20" t="s">
-        <v>3481</v>
       </c>
       <c r="G44" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B44 ) &gt; 0, "OK", "KO" )</f>
@@ -62666,16 +62667,16 @@
         <v>3402</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>3482</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F45" s="20" t="s">
         <v>3483</v>
-      </c>
-      <c r="D45" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F45" s="20" t="s">
-        <v>3484</v>
       </c>
       <c r="G45" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B45 ) &gt; 0, "OK", "KO" )</f>
@@ -62684,19 +62685,19 @@
     </row>
     <row r="46" spans="2:7">
       <c r="B46" s="14" t="s">
-        <v>3485</v>
+        <v>3484</v>
       </c>
       <c r="C46" s="14" t="s">
+        <v>3482</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F46" s="20" t="s">
         <v>3483</v>
-      </c>
-      <c r="D46" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E46" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F46" s="20" t="s">
-        <v>3484</v>
       </c>
       <c r="G46" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B46 ) &gt; 0, "OK", "KO" )</f>
@@ -62708,16 +62709,16 @@
         <v>3358</v>
       </c>
       <c r="C47" s="14" t="s">
+        <v>3485</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E47" s="14" t="s">
         <v>3486</v>
       </c>
-      <c r="D47" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E47" s="14" t="s">
+      <c r="F47" s="20" t="s">
         <v>3487</v>
-      </c>
-      <c r="F47" s="20" t="s">
-        <v>3488</v>
       </c>
       <c r="G47" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B47 ) &gt; 0, "OK", "KO" )</f>
@@ -62729,16 +62730,16 @@
         <v>3358</v>
       </c>
       <c r="C48" s="14" t="s">
+        <v>3488</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>3486</v>
+      </c>
+      <c r="F48" s="20" t="s">
         <v>3489</v>
-      </c>
-      <c r="D48" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>3487</v>
-      </c>
-      <c r="F48" s="20" t="s">
-        <v>3490</v>
       </c>
       <c r="G48" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B48 ) &gt; 0, "OK", "KO" )</f>
@@ -62750,16 +62751,16 @@
         <v>3365</v>
       </c>
       <c r="C49" s="14" t="s">
+        <v>3490</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>3486</v>
+      </c>
+      <c r="F49" s="20" t="s">
         <v>3491</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>3487</v>
-      </c>
-      <c r="F49" s="20" t="s">
-        <v>3492</v>
       </c>
       <c r="G49" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B49 ) &gt; 0, "OK", "KO" )</f>
@@ -62771,16 +62772,16 @@
         <v>3371</v>
       </c>
       <c r="C50" s="14" t="s">
+        <v>3492</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E50" s="14" t="s">
         <v>3493</v>
       </c>
-      <c r="D50" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E50" s="14" t="s">
+      <c r="F50" s="20" t="s">
         <v>3494</v>
-      </c>
-      <c r="F50" s="20" t="s">
-        <v>3495</v>
       </c>
       <c r="G50" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B50 ) &gt; 0, "OK", "KO" )</f>
@@ -62792,16 +62793,16 @@
         <v>3383</v>
       </c>
       <c r="C51" s="14" t="s">
+        <v>3495</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F51" s="20" t="s">
         <v>3496</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F51" s="20" t="s">
-        <v>3497</v>
       </c>
       <c r="G51" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B51 ) &gt; 0, "OK", "KO" )</f>
@@ -62813,16 +62814,16 @@
         <v>3404</v>
       </c>
       <c r="C52" s="14" t="s">
+        <v>3497</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F52" s="20" t="s">
         <v>3498</v>
-      </c>
-      <c r="D52" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E52" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F52" s="20" t="s">
-        <v>3499</v>
       </c>
       <c r="G52" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B52 ) &gt; 0, "OK", "KO" )</f>
@@ -62834,16 +62835,16 @@
         <v>3395</v>
       </c>
       <c r="C53" s="14" t="s">
+        <v>3497</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F53" s="20" t="s">
         <v>3498</v>
-      </c>
-      <c r="D53" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F53" s="20" t="s">
-        <v>3499</v>
       </c>
       <c r="G53" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B53 ) &gt; 0, "OK", "KO" )</f>
@@ -62855,16 +62856,16 @@
         <v>3395</v>
       </c>
       <c r="C54" s="14" t="s">
+        <v>3499</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F54" s="20" t="s">
         <v>3500</v>
-      </c>
-      <c r="D54" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E54" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F54" s="20" t="s">
-        <v>3501</v>
       </c>
       <c r="G54" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B54 ) &gt; 0, "OK", "KO" )</f>
@@ -62876,16 +62877,16 @@
         <v>3368</v>
       </c>
       <c r="C55" s="14" t="s">
+        <v>3501</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F55" s="20" t="s">
         <v>3502</v>
-      </c>
-      <c r="D55" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E55" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F55" s="20" t="s">
-        <v>3503</v>
       </c>
       <c r="G55" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B55 ) &gt; 0, "OK", "KO" )</f>
@@ -62897,16 +62898,16 @@
         <v>3368</v>
       </c>
       <c r="C56" s="14" t="s">
+        <v>3503</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F56" s="20" t="s">
         <v>3504</v>
-      </c>
-      <c r="D56" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E56" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F56" s="20" t="s">
-        <v>3505</v>
       </c>
       <c r="G56" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B56 ) &gt; 0, "OK", "KO" )</f>
@@ -62918,16 +62919,16 @@
         <v>3372</v>
       </c>
       <c r="C57" s="14" t="s">
+        <v>3505</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E57" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F57" s="20" t="s">
         <v>3506</v>
-      </c>
-      <c r="D57" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E57" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F57" s="20" t="s">
-        <v>3507</v>
       </c>
       <c r="G57" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B57 ) &gt; 0, "OK", "KO" )</f>
@@ -62939,16 +62940,16 @@
         <v>3389</v>
       </c>
       <c r="C58" s="14" t="s">
+        <v>3536</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E58" s="14" t="s">
         <v>3537</v>
       </c>
-      <c r="D58" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E58" s="14" t="s">
+      <c r="F58" s="20" t="s">
         <v>3538</v>
-      </c>
-      <c r="F58" s="20" t="s">
-        <v>3539</v>
       </c>
       <c r="G58" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B58 ) &gt; 0, "OK", "KO" )</f>
@@ -62960,16 +62961,16 @@
         <v>3389</v>
       </c>
       <c r="C59" s="14" t="s">
+        <v>3539</v>
+      </c>
+      <c r="D59" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E59" s="14" t="s">
         <v>3540</v>
       </c>
-      <c r="D59" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E59" s="14" t="s">
+      <c r="F59" s="20" t="s">
         <v>3541</v>
-      </c>
-      <c r="F59" s="20" t="s">
-        <v>3542</v>
       </c>
       <c r="G59" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B59 ) &gt; 0, "OK", "KO" )</f>
@@ -62981,16 +62982,16 @@
         <v>3366</v>
       </c>
       <c r="C60" s="14" t="s">
+        <v>3466</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E60" s="14" t="s">
+        <v>3463</v>
+      </c>
+      <c r="F60" s="20" t="s">
         <v>3467</v>
-      </c>
-      <c r="D60" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E60" s="14" t="s">
-        <v>3464</v>
-      </c>
-      <c r="F60" s="20" t="s">
-        <v>3468</v>
       </c>
       <c r="G60" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B60 ) &gt; 0, "OK", "KO" )</f>
@@ -63023,7 +63024,7 @@
         <v>3377</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="D62" s="14" t="s">
         <v>3449</v>
@@ -63032,7 +63033,7 @@
         <v>3450</v>
       </c>
       <c r="F62" s="20" t="s">
-        <v>3547</v>
+        <v>3546</v>
       </c>
       <c r="G62" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B62 ) &gt; 0, "OK", "KO" )</f>
@@ -63065,16 +63066,16 @@
         <v>3373</v>
       </c>
       <c r="C64" s="14" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D64" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E64" s="14" t="s">
+        <v>3475</v>
+      </c>
+      <c r="F64" s="20" t="s">
         <v>3480</v>
-      </c>
-      <c r="D64" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E64" s="14" t="s">
-        <v>3476</v>
-      </c>
-      <c r="F64" s="20" t="s">
-        <v>3481</v>
       </c>
       <c r="G64" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B64 ) &gt; 0, "OK", "KO" )</f>
@@ -63086,16 +63087,16 @@
         <v>3374</v>
       </c>
       <c r="C65" s="14" t="s">
+        <v>3471</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E65" s="14" t="s">
+        <v>3469</v>
+      </c>
+      <c r="F65" s="20" t="s">
         <v>3472</v>
-      </c>
-      <c r="D65" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E65" s="14" t="s">
-        <v>3470</v>
-      </c>
-      <c r="F65" s="20" t="s">
-        <v>3473</v>
       </c>
       <c r="G65" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B65 ) &gt; 0, "OK", "KO" )</f>
@@ -63107,16 +63108,16 @@
         <v>3378</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>3548</v>
+        <v>3547</v>
       </c>
       <c r="D66" s="14" t="s">
         <v>3432</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="F66" s="20" t="s">
-        <v>3549</v>
+        <v>3548</v>
       </c>
       <c r="G66" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B66 ) &gt; 0, "OK", "KO" )</f>
@@ -63128,7 +63129,7 @@
         <v>3379</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>3552</v>
+        <v>3551</v>
       </c>
       <c r="D67" s="14" t="s">
         <v>3449</v>
@@ -63137,7 +63138,7 @@
         <v>3457</v>
       </c>
       <c r="F67" s="20" t="s">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="G67" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B67 ) &gt; 0, "OK", "KO" )</f>
@@ -63149,16 +63150,16 @@
         <v>3388</v>
       </c>
       <c r="C68" s="14" t="s">
+        <v>3525</v>
+      </c>
+      <c r="D68" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E68" s="14" t="s">
+        <v>3463</v>
+      </c>
+      <c r="F68" s="20" t="s">
         <v>3526</v>
-      </c>
-      <c r="D68" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E68" s="14" t="s">
-        <v>3464</v>
-      </c>
-      <c r="F68" s="20" t="s">
-        <v>3527</v>
       </c>
       <c r="G68" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B68 ) &gt; 0, "OK", "KO" )</f>
@@ -63170,16 +63171,16 @@
         <v>3388</v>
       </c>
       <c r="C69" s="14" t="s">
+        <v>3527</v>
+      </c>
+      <c r="D69" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E69" s="14" t="s">
+        <v>3469</v>
+      </c>
+      <c r="F69" s="20" t="s">
         <v>3528</v>
-      </c>
-      <c r="D69" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E69" s="14" t="s">
-        <v>3470</v>
-      </c>
-      <c r="F69" s="20" t="s">
-        <v>3529</v>
       </c>
       <c r="G69" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B69 ) &gt; 0, "OK", "KO" )</f>
@@ -63191,7 +63192,7 @@
         <v>3388</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>3530</v>
+        <v>3529</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>3449</v>
@@ -63200,7 +63201,7 @@
         <v>3450</v>
       </c>
       <c r="F70" s="20" t="s">
-        <v>3531</v>
+        <v>3530</v>
       </c>
       <c r="G70" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B70 ) &gt; 0, "OK", "KO" )</f>
@@ -63212,16 +63213,16 @@
         <v>3388</v>
       </c>
       <c r="C71" s="14" t="s">
+        <v>3531</v>
+      </c>
+      <c r="D71" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E71" s="14" t="s">
+        <v>3493</v>
+      </c>
+      <c r="F71" s="20" t="s">
         <v>3532</v>
-      </c>
-      <c r="D71" s="14" t="s">
-        <v>3475</v>
-      </c>
-      <c r="E71" s="14" t="s">
-        <v>3494</v>
-      </c>
-      <c r="F71" s="20" t="s">
-        <v>3533</v>
       </c>
       <c r="G71" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B71 ) &gt; 0, "OK", "KO" )</f>
@@ -63233,16 +63234,16 @@
         <v>3388</v>
       </c>
       <c r="C72" s="14" t="s">
+        <v>3533</v>
+      </c>
+      <c r="D72" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>3463</v>
+      </c>
+      <c r="F72" s="20" t="s">
         <v>3534</v>
-      </c>
-      <c r="D72" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E72" s="14" t="s">
-        <v>3464</v>
-      </c>
-      <c r="F72" s="20" t="s">
-        <v>3535</v>
       </c>
       <c r="G72" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B72 ) &gt; 0, "OK", "KO" )</f>
@@ -63254,16 +63255,16 @@
         <v>3396</v>
       </c>
       <c r="C73" s="14" t="s">
+        <v>3464</v>
+      </c>
+      <c r="D73" s="14" t="s">
+        <v>3575</v>
+      </c>
+      <c r="E73" s="14" t="s">
         <v>3465</v>
       </c>
-      <c r="D73" s="14" t="s">
-        <v>3463</v>
-      </c>
-      <c r="E73" s="14" t="s">
-        <v>3466</v>
-      </c>
       <c r="F73" s="20" t="s">
-        <v>3573</v>
+        <v>3572</v>
       </c>
       <c r="G73" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B73 ) &gt; 0, "OK", "KO" )</f>
@@ -63275,16 +63276,16 @@
         <v>3397</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>3572</v>
+        <v>3571</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>3475</v>
+        <v>3474</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>3494</v>
+        <v>3493</v>
       </c>
       <c r="F74" s="20" t="s">
-        <v>3551</v>
+        <v>3550</v>
       </c>
       <c r="G74" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B74 ) &gt; 0, "OK", "KO" )</f>
@@ -63296,16 +63297,16 @@
         <v>3398</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="D75" s="14" t="s">
-        <v>3463</v>
+        <v>3575</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>3466</v>
+        <v>3465</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>3543</v>
+        <v>3542</v>
       </c>
       <c r="G75" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B75 ) &gt; 0, "OK", "KO" )</f>
@@ -63317,7 +63318,7 @@
         <v>3398</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>3544</v>
+        <v>3543</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>3413</v>
@@ -63326,7 +63327,7 @@
         <v>3414</v>
       </c>
       <c r="F76" s="20" t="s">
-        <v>3545</v>
+        <v>3544</v>
       </c>
       <c r="G76" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B76 ) &gt; 0, "OK", "KO" )</f>
@@ -63359,7 +63360,7 @@
         <v>3405</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>3554</v>
+        <v>3553</v>
       </c>
       <c r="D78" s="14" t="s">
         <v>3449</v>
@@ -63368,7 +63369,7 @@
         <v>3450</v>
       </c>
       <c r="F78" s="20" t="s">
-        <v>3555</v>
+        <v>3554</v>
       </c>
       <c r="G78" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B78 ) &gt; 0, "OK", "KO" )</f>
@@ -63380,16 +63381,16 @@
         <v>3393</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="D79" s="14" t="s">
+        <v>3474</v>
+      </c>
+      <c r="E79" s="14" t="s">
         <v>3475</v>
       </c>
-      <c r="E79" s="14" t="s">
-        <v>3476</v>
-      </c>
       <c r="F79" s="20" t="s">
-        <v>3558</v>
+        <v>3557</v>
       </c>
       <c r="G79" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B79 ) &gt; 0, "OK", "KO" )</f>
@@ -63401,16 +63402,16 @@
         <v>3357</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>3550</v>
+        <v>3549</v>
       </c>
       <c r="D80" s="14" t="s">
-        <v>3475</v>
+        <v>3474</v>
       </c>
       <c r="E80" s="14" t="s">
-        <v>3494</v>
+        <v>3493</v>
       </c>
       <c r="F80" s="20" t="s">
-        <v>3559</v>
+        <v>3558</v>
       </c>
       <c r="G80" s="21" t="str">
         <f>IF( COUNTIF( Papers!A:A,  B80 ) &gt; 0, "OK", "KO" )</f>
@@ -66205,7 +66206,7 @@
     <row r="1" spans="1:9">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>3560</v>
+        <v>3559</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -66214,15 +66215,15 @@
       <c r="G2" s="23"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="B4" s="38" t="s">
-        <v>3561</v>
-      </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="40">
+      <c r="B4" s="42" t="s">
+        <v>3560</v>
+      </c>
+      <c r="C4" s="43"/>
+      <c r="D4" s="44">
         <f>COUNTA( Papers!C:C ) - 1</f>
         <v>599</v>
       </c>
-      <c r="E4" s="39"/>
+      <c r="E4" s="43"/>
     </row>
     <row r="5" spans="1:9">
       <c r="C5" s="23"/>
@@ -66235,10 +66236,10 @@
     <row r="6" spans="1:9">
       <c r="C6" s="23"/>
       <c r="D6" s="24" t="s">
+        <v>3561</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>3562</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>3563</v>
       </c>
       <c r="F6" s="23"/>
       <c r="G6" s="23"/>
@@ -66246,11 +66247,11 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="26"/>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="45" t="s">
+        <v>3563</v>
+      </c>
+      <c r="C7" s="27" t="s">
         <v>3564</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>3565</v>
       </c>
       <c r="D7" s="28">
         <f>COUNTIF( Papers!E:E, "Yes" )</f>
@@ -66266,9 +66267,9 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="26"/>
-      <c r="B8" s="42"/>
+      <c r="B8" s="46"/>
       <c r="C8" s="30" t="s">
-        <v>3566</v>
+        <v>3565</v>
       </c>
       <c r="D8" s="19">
         <f>COUNTIF( Papers!E:E, "No" )</f>
@@ -66284,26 +66285,26 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="26"/>
-      <c r="B9" s="43"/>
+      <c r="B9" s="47"/>
       <c r="C9" s="32" t="s">
-        <v>3567</v>
-      </c>
-      <c r="D9" s="44" t="str">
+        <v>3566</v>
+      </c>
+      <c r="D9" s="40" t="str">
         <f>IF(SUM(D7:D8)=$D$4,"OK","KO")</f>
         <v>OK</v>
       </c>
-      <c r="E9" s="45"/>
+      <c r="E9" s="41"/>
       <c r="G9" s="1" t="s">
         <v>3361</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="26"/>
-      <c r="B10" s="46" t="s">
-        <v>3574</v>
+      <c r="B10" s="37" t="s">
+        <v>3573</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>3565</v>
+        <v>3564</v>
       </c>
       <c r="D10" s="28">
         <f>COUNTIF( Papers!F:F, "Yes" )</f>
@@ -66316,9 +66317,9 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="26"/>
-      <c r="B11" s="47"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="30" t="s">
-        <v>3566</v>
+        <v>3565</v>
       </c>
       <c r="D11" s="19">
         <f>COUNTIF( Papers!F:F, "No" )</f>
@@ -66331,22 +66332,22 @@
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1">
       <c r="A12" s="26"/>
-      <c r="B12" s="48"/>
+      <c r="B12" s="39"/>
       <c r="C12" s="32" t="s">
-        <v>3567</v>
-      </c>
-      <c r="D12" s="44" t="str">
+        <v>3566</v>
+      </c>
+      <c r="D12" s="40" t="str">
         <f>IF(SUM(D10:D11)=$D$4,"OK","KO")</f>
         <v>OK</v>
       </c>
-      <c r="E12" s="45"/>
+      <c r="E12" s="41"/>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1" thickTop="1">
-      <c r="B13" s="46" t="s">
-        <v>3575</v>
+      <c r="B13" s="37" t="s">
+        <v>3574</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>3565</v>
+        <v>3564</v>
       </c>
       <c r="D13" s="28">
         <f>COUNTIFS( Papers!E:E, "Yes", Papers!F:F, "Yes" )</f>
@@ -66356,12 +66357,12 @@
         <f>D13/$D$7</f>
         <v>0.17669172932330826</v>
       </c>
-      <c r="I13" s="49"/>
+      <c r="I13" s="36"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="B14" s="47"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="30" t="s">
-        <v>3566</v>
+        <v>3565</v>
       </c>
       <c r="D14" s="19">
         <f>COUNTIFS( Papers!E:E, "Yes", Papers!F:F, "No" )</f>
@@ -66371,24 +66372,24 @@
         <f>D14/$D$7</f>
         <v>0.82330827067669177</v>
       </c>
-      <c r="I14" s="49"/>
+      <c r="I14" s="36"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1">
-      <c r="B15" s="48"/>
+      <c r="B15" s="39"/>
       <c r="C15" s="32" t="s">
-        <v>3567</v>
-      </c>
-      <c r="D15" s="44" t="str">
+        <v>3566</v>
+      </c>
+      <c r="D15" s="40" t="str">
         <f>IF(SUM(D13:D14)=$D$7,"OK","KO")</f>
         <v>OK</v>
       </c>
-      <c r="E15" s="45"/>
+      <c r="E15" s="41"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickTop="1"/>
     <row r="17" spans="3:5" ht="15.75" thickBot="1"/>
     <row r="18" spans="3:5" ht="15" customHeight="1" thickTop="1">
       <c r="C18" s="33" t="s">
-        <v>3568</v>
+        <v>3567</v>
       </c>
       <c r="D18" s="28">
         <f>COUNTIFS(    Papers!F:F, "Yes",  Papers!D:D, G7  )</f>
@@ -66401,7 +66402,7 @@
     </row>
     <row r="19" spans="3:5" ht="15" customHeight="1">
       <c r="C19" s="34" t="s">
-        <v>3569</v>
+        <v>3568</v>
       </c>
       <c r="D19" s="19">
         <f>COUNTIFS(    Papers!F:F, "Yes",  Papers!D:D, G8  )</f>
@@ -66414,7 +66415,7 @@
     </row>
     <row r="20" spans="3:5" ht="15" customHeight="1">
       <c r="C20" s="34" t="s">
-        <v>3570</v>
+        <v>3569</v>
       </c>
       <c r="D20" s="19">
         <f>COUNTIFS(    Papers!F:F, "Yes",  Papers!D:D, G9  )</f>
@@ -66427,13 +66428,13 @@
     </row>
     <row r="21" spans="3:5" ht="15" customHeight="1" thickBot="1">
       <c r="C21" s="35" t="s">
-        <v>3567</v>
-      </c>
-      <c r="D21" s="44" t="str">
+        <v>3566</v>
+      </c>
+      <c r="D21" s="40" t="str">
         <f>IF(SUM(D18:D20)=D10,"OK","KO")</f>
         <v>OK</v>
       </c>
-      <c r="E21" s="45"/>
+      <c r="E21" s="41"/>
     </row>
     <row r="22" spans="3:5" ht="15" customHeight="1" thickTop="1"/>
   </sheetData>
@@ -66463,7 +66464,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" s="1" t="s">
-        <v>3571</v>
+        <v>3570</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>